<commit_message>
feat: add Gift City Relitrade Salary Data Excel file to HRMS documentation
</commit_message>
<xml_diff>
--- a/docs/HRMS x Sanghvi Association/Gift City Relitrade Salary Data.xlsx
+++ b/docs/HRMS x Sanghvi Association/Gift City Relitrade Salary Data.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manish.kandel\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\manish.kandel\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AD852E2F-2E2F-4130-9B75-0FDB20CD5B08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CC16D17F-F535-4903-BB2B-E2A36BDAA603}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0F8B3EAC-F07F-4CA5-A8D8-BEA9EBE60320}"/>
   </bookViews>
@@ -115,9 +115,6 @@
     <t>PAYABLE GROSS</t>
   </si>
   <si>
-    <t>NET PAYABLE</t>
-  </si>
-  <si>
     <t>EMPLOYEE
 ESIC</t>
   </si>
@@ -138,6 +135,9 @@
   </si>
   <si>
     <t>Totals</t>
+  </si>
+  <si>
+    <t>NET PAYABLE</t>
   </si>
 </sst>
 </file>
@@ -145,9 +145,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
-    <numFmt numFmtId="167" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="168" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="169" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="165" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
@@ -256,11 +256,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -268,7 +269,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="17" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -277,7 +278,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -287,58 +288,31 @@
     <xf numFmtId="17" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="3" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="5" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="3" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="5" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="168" fontId="5" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="168" fontId="5" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="5" fillId="3" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Comma" xfId="2" builtinId="3"/>
     <cellStyle name="Comma 2" xfId="1" xr:uid="{F80F9DF9-EA98-4FCD-A2BD-91A222B3046C}"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -678,7 +652,8 @@
     <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5546875" style="11" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" customWidth="1"/>
+    <col min="13" max="13" width="11.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="46.8" x14ac:dyDescent="0.3">
@@ -697,29 +672,29 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="F1" s="11" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="H1" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="I1" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="I1" s="23" t="s">
+      <c r="J1" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="J1" s="23" t="s">
-        <v>29</v>
-      </c>
-      <c r="K1" s="30" t="s">
+      <c r="K1" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="L1" s="36" t="s">
+      <c r="L1" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="M1" s="43" t="s">
-        <v>24</v>
+      <c r="M1" s="11" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
@@ -738,24 +713,24 @@
       <c r="E2" s="6">
         <v>45273</v>
       </c>
-      <c r="F2" s="16">
+      <c r="F2" s="14">
         <v>130</v>
       </c>
-      <c r="G2" s="16"/>
-      <c r="H2" s="17">
+      <c r="G2" s="14"/>
+      <c r="H2" s="15">
         <v>200</v>
       </c>
-      <c r="I2" s="25">
+      <c r="I2" s="14">
         <v>563</v>
       </c>
-      <c r="J2" s="25"/>
-      <c r="K2" s="33">
+      <c r="J2" s="14"/>
+      <c r="K2" s="23">
         <v>17330</v>
       </c>
-      <c r="L2" s="40">
+      <c r="L2" s="23">
         <v>17330</v>
       </c>
-      <c r="M2" s="45">
+      <c r="M2" s="25">
         <v>17000</v>
       </c>
     </row>
@@ -775,24 +750,24 @@
       <c r="E3" s="10">
         <v>45309</v>
       </c>
-      <c r="F3" s="18">
+      <c r="F3" s="16">
         <v>120</v>
       </c>
-      <c r="G3" s="18"/>
-      <c r="H3" s="19">
+      <c r="G3" s="16"/>
+      <c r="H3" s="17">
         <v>200</v>
       </c>
-      <c r="I3" s="26">
+      <c r="I3" s="16">
         <v>519</v>
       </c>
-      <c r="J3" s="26"/>
-      <c r="K3" s="34">
+      <c r="J3" s="16"/>
+      <c r="K3" s="7">
         <v>15980</v>
       </c>
-      <c r="L3" s="41">
+      <c r="L3" s="7">
         <v>15980</v>
       </c>
-      <c r="M3" s="45">
+      <c r="M3" s="25">
         <v>15660</v>
       </c>
     </row>
@@ -812,25 +787,25 @@
       <c r="E4" s="6">
         <v>45691</v>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="14">
         <v>0</v>
       </c>
-      <c r="G4" s="16"/>
-      <c r="H4" s="17">
+      <c r="G4" s="14"/>
+      <c r="H4" s="15">
         <v>200</v>
       </c>
-      <c r="I4" s="25">
+      <c r="I4" s="14">
         <v>0</v>
       </c>
-      <c r="J4" s="25"/>
-      <c r="K4" s="33">
+      <c r="J4" s="14"/>
+      <c r="K4" s="23">
         <v>150000</v>
       </c>
-      <c r="L4" s="40">
+      <c r="L4" s="23">
         <v>150000</v>
       </c>
-      <c r="M4" s="45">
-        <v>273132</v>
+      <c r="M4" s="25">
+        <v>149800</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
@@ -849,25 +824,25 @@
       <c r="E5" s="6">
         <v>45792</v>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="14">
         <v>0</v>
       </c>
-      <c r="G5" s="16"/>
-      <c r="H5" s="17">
+      <c r="G5" s="14"/>
+      <c r="H5" s="15">
         <v>200</v>
       </c>
-      <c r="I5" s="25">
+      <c r="I5" s="14">
         <v>0</v>
       </c>
-      <c r="J5" s="25"/>
-      <c r="K5" s="33">
+      <c r="J5" s="14"/>
+      <c r="K5" s="23">
         <v>32000</v>
       </c>
-      <c r="L5" s="40">
+      <c r="L5" s="23">
         <v>32000</v>
       </c>
-      <c r="M5" s="45">
-        <v>63400</v>
+      <c r="M5" s="25">
+        <v>31800</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
@@ -886,24 +861,24 @@
       <c r="E6" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="18">
+      <c r="F6" s="16">
         <v>0</v>
       </c>
-      <c r="G6" s="18"/>
-      <c r="H6" s="19">
+      <c r="G6" s="16"/>
+      <c r="H6" s="17">
         <v>200</v>
       </c>
-      <c r="I6" s="26">
+      <c r="I6" s="16">
         <v>0</v>
       </c>
-      <c r="J6" s="26"/>
-      <c r="K6" s="34">
+      <c r="J6" s="16"/>
+      <c r="K6" s="7">
         <v>37500</v>
       </c>
-      <c r="L6" s="41">
+      <c r="L6" s="7">
         <v>37500</v>
       </c>
-      <c r="M6" s="46">
+      <c r="M6" s="26">
         <v>33550</v>
       </c>
     </row>
@@ -923,24 +898,24 @@
       <c r="E7" s="3">
         <v>46023</v>
       </c>
-      <c r="F7" s="15">
+      <c r="F7" s="13">
         <v>0</v>
       </c>
-      <c r="G7" s="15"/>
-      <c r="H7" s="14">
+      <c r="G7" s="13"/>
+      <c r="H7" s="12">
         <v>200</v>
       </c>
-      <c r="I7" s="24">
+      <c r="I7" s="13">
         <v>0</v>
       </c>
-      <c r="J7" s="24"/>
-      <c r="K7" s="31">
+      <c r="J7" s="13"/>
+      <c r="K7" s="21">
         <v>30000</v>
       </c>
-      <c r="L7" s="37">
+      <c r="L7" s="21">
         <v>30000</v>
       </c>
-      <c r="M7" s="45">
+      <c r="M7" s="25">
         <v>26800</v>
       </c>
     </row>
@@ -960,28 +935,28 @@
       <c r="E8" s="3">
         <v>46023</v>
       </c>
-      <c r="F8" s="15">
+      <c r="F8" s="13">
         <v>113</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="13">
         <v>906</v>
       </c>
-      <c r="H8" s="14">
+      <c r="H8" s="12">
         <v>200</v>
       </c>
-      <c r="I8" s="24">
+      <c r="I8" s="13">
         <v>491</v>
       </c>
-      <c r="J8" s="24">
+      <c r="J8" s="13">
         <v>906</v>
       </c>
-      <c r="K8" s="31">
+      <c r="K8" s="21">
         <v>15103</v>
       </c>
-      <c r="L8" s="37">
+      <c r="L8" s="21">
         <v>15103</v>
       </c>
-      <c r="M8" s="45">
+      <c r="M8" s="25">
         <v>13884</v>
       </c>
     </row>
@@ -1001,98 +976,66 @@
       <c r="E9" s="10">
         <v>45810</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="16">
         <v>109</v>
       </c>
-      <c r="G9" s="20"/>
-      <c r="H9" s="19">
+      <c r="G9" s="18"/>
+      <c r="H9" s="17">
         <v>200</v>
       </c>
-      <c r="I9" s="26">
+      <c r="I9" s="16">
         <v>472</v>
       </c>
-      <c r="J9" s="27"/>
-      <c r="K9" s="34">
+      <c r="J9" s="18"/>
+      <c r="K9" s="7">
         <v>14530</v>
       </c>
-      <c r="L9" s="41">
+      <c r="L9" s="7">
         <v>14530</v>
       </c>
-      <c r="M9" s="45">
+      <c r="M9" s="25">
         <v>14221</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" s="44" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" s="44"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="28"/>
-      <c r="H10" s="28"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="44"/>
-      <c r="K10" s="32">
+      <c r="A10" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="20"/>
+      <c r="H10" s="20"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22">
         <v>312443</v>
       </c>
-      <c r="L10" s="38">
+      <c r="L10" s="22">
         <v>312443</v>
       </c>
-      <c r="M10" s="44">
-        <v>457647</v>
+      <c r="M10" s="22">
+        <f t="shared" ref="M10" si="0">SUM(M2:M9)</f>
+        <v>302715</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="21"/>
-      <c r="I11" s="22"/>
-      <c r="J11" s="22"/>
+      <c r="H11" s="19"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="21"/>
-      <c r="I12" s="22"/>
-      <c r="J12" s="22"/>
-      <c r="K12" s="29"/>
-      <c r="L12" s="35"/>
-      <c r="M12" s="42"/>
+      <c r="H12" s="19"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="21"/>
-      <c r="I13" s="22"/>
-      <c r="J13" s="22"/>
-      <c r="K13" s="29"/>
-      <c r="L13" s="35"/>
-      <c r="M13" s="47"/>
+      <c r="H13" s="19"/>
+      <c r="M13" s="27"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="22"/>
-      <c r="J14" s="22"/>
-      <c r="K14" s="29"/>
-      <c r="L14" s="35"/>
-      <c r="M14" s="42"/>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="I15" s="22"/>
-      <c r="J15" s="22"/>
-      <c r="K15" s="29"/>
-      <c r="L15" s="35"/>
-      <c r="M15" s="42"/>
+      <c r="H14" s="19"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="K16" s="29"/>
-      <c r="L16" s="39"/>
-      <c r="M16" s="42"/>
+      <c r="L16" s="24"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>